<commit_message>
Excel corso invalidità civile: aggiungi riepilogo mensile automatico e 60 righe per sezione
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UJqD5pkzvn9qNWWBae35Bo
</commit_message>
<xml_diff>
--- a/Corso_Invalidita_Civile_Ottobre_2026.xlsx
+++ b/Corso_Invalidita_Civile_Ottobre_2026.xlsx
@@ -16,13 +16,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.00 &quot;€&quot;;[Red]-#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="168" formatCode="MMMM YYYY"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,8 +80,17 @@
     <font>
       <color rgb="002E7D32"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +122,16 @@
         <fgColor rgb="00E3F4E4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -181,6 +201,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -580,7 +620,7 @@
         </is>
       </c>
       <c r="C4" s="4">
-        <f>SUM(C8:C37)</f>
+        <f>SUM(C8:C67)</f>
         <v/>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -600,7 +640,7 @@
         </is>
       </c>
       <c r="C5" s="8">
-        <f>SUM(H8:H37)</f>
+        <f>SUM(H8:H67)</f>
         <v/>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -609,7 +649,7 @@
         </is>
       </c>
       <c r="F5" s="9">
-        <f>SUM(G8:G37)</f>
+        <f>SUM(G8:G67)</f>
         <v/>
       </c>
     </row>
@@ -939,16 +979,614 @@
       <c r="G37" s="19" t="n"/>
       <c r="H37" s="20" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="14" t="n"/>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="16" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="19" t="n"/>
+      <c r="H38" s="20" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="n"/>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="16" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="18" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="20" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="n"/>
+      <c r="B40" s="15" t="n"/>
+      <c r="C40" s="16" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="18" t="n"/>
+      <c r="G40" s="19" t="n"/>
+      <c r="H40" s="20" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="n"/>
+      <c r="B41" s="15" t="n"/>
+      <c r="C41" s="16" t="n"/>
+      <c r="E41" s="17" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="19" t="n"/>
+      <c r="H41" s="20" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="n"/>
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="16" t="n"/>
+      <c r="E42" s="17" t="n"/>
+      <c r="F42" s="18" t="n"/>
+      <c r="G42" s="19" t="n"/>
+      <c r="H42" s="20" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="n"/>
+      <c r="B43" s="15" t="n"/>
+      <c r="C43" s="16" t="n"/>
+      <c r="E43" s="17" t="n"/>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="19" t="n"/>
+      <c r="H43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="n"/>
+      <c r="B44" s="15" t="n"/>
+      <c r="C44" s="16" t="n"/>
+      <c r="E44" s="17" t="n"/>
+      <c r="F44" s="18" t="n"/>
+      <c r="G44" s="19" t="n"/>
+      <c r="H44" s="20" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="n"/>
+      <c r="B45" s="15" t="n"/>
+      <c r="C45" s="16" t="n"/>
+      <c r="E45" s="17" t="n"/>
+      <c r="F45" s="18" t="n"/>
+      <c r="G45" s="19" t="n"/>
+      <c r="H45" s="20" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="n"/>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="16" t="n"/>
+      <c r="E46" s="17" t="n"/>
+      <c r="F46" s="18" t="n"/>
+      <c r="G46" s="19" t="n"/>
+      <c r="H46" s="20" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="n"/>
+      <c r="B47" s="15" t="n"/>
+      <c r="C47" s="16" t="n"/>
+      <c r="E47" s="17" t="n"/>
+      <c r="F47" s="18" t="n"/>
+      <c r="G47" s="19" t="n"/>
+      <c r="H47" s="20" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="n"/>
+      <c r="B48" s="15" t="n"/>
+      <c r="C48" s="16" t="n"/>
+      <c r="E48" s="17" t="n"/>
+      <c r="F48" s="18" t="n"/>
+      <c r="G48" s="19" t="n"/>
+      <c r="H48" s="20" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="n"/>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="16" t="n"/>
+      <c r="E49" s="17" t="n"/>
+      <c r="F49" s="18" t="n"/>
+      <c r="G49" s="19" t="n"/>
+      <c r="H49" s="20" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="n"/>
+      <c r="B50" s="15" t="n"/>
+      <c r="C50" s="16" t="n"/>
+      <c r="E50" s="17" t="n"/>
+      <c r="F50" s="18" t="n"/>
+      <c r="G50" s="19" t="n"/>
+      <c r="H50" s="20" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="n"/>
+      <c r="B51" s="15" t="n"/>
+      <c r="C51" s="16" t="n"/>
+      <c r="E51" s="17" t="n"/>
+      <c r="F51" s="18" t="n"/>
+      <c r="G51" s="19" t="n"/>
+      <c r="H51" s="20" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="n"/>
+      <c r="B52" s="15" t="n"/>
+      <c r="C52" s="16" t="n"/>
+      <c r="E52" s="17" t="n"/>
+      <c r="F52" s="18" t="n"/>
+      <c r="G52" s="19" t="n"/>
+      <c r="H52" s="20" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="n"/>
+      <c r="B53" s="15" t="n"/>
+      <c r="C53" s="16" t="n"/>
+      <c r="E53" s="17" t="n"/>
+      <c r="F53" s="18" t="n"/>
+      <c r="G53" s="19" t="n"/>
+      <c r="H53" s="20" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="n"/>
+      <c r="B54" s="15" t="n"/>
+      <c r="C54" s="16" t="n"/>
+      <c r="E54" s="17" t="n"/>
+      <c r="F54" s="18" t="n"/>
+      <c r="G54" s="19" t="n"/>
+      <c r="H54" s="20" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="n"/>
+      <c r="B55" s="15" t="n"/>
+      <c r="C55" s="16" t="n"/>
+      <c r="E55" s="17" t="n"/>
+      <c r="F55" s="18" t="n"/>
+      <c r="G55" s="19" t="n"/>
+      <c r="H55" s="20" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="n"/>
+      <c r="B56" s="15" t="n"/>
+      <c r="C56" s="16" t="n"/>
+      <c r="E56" s="17" t="n"/>
+      <c r="F56" s="18" t="n"/>
+      <c r="G56" s="19" t="n"/>
+      <c r="H56" s="20" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="n"/>
+      <c r="B57" s="15" t="n"/>
+      <c r="C57" s="16" t="n"/>
+      <c r="E57" s="17" t="n"/>
+      <c r="F57" s="18" t="n"/>
+      <c r="G57" s="19" t="n"/>
+      <c r="H57" s="20" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="n"/>
+      <c r="B58" s="15" t="n"/>
+      <c r="C58" s="16" t="n"/>
+      <c r="E58" s="17" t="n"/>
+      <c r="F58" s="18" t="n"/>
+      <c r="G58" s="19" t="n"/>
+      <c r="H58" s="20" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="n"/>
+      <c r="B59" s="15" t="n"/>
+      <c r="C59" s="16" t="n"/>
+      <c r="E59" s="17" t="n"/>
+      <c r="F59" s="18" t="n"/>
+      <c r="G59" s="19" t="n"/>
+      <c r="H59" s="20" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="n"/>
+      <c r="B60" s="15" t="n"/>
+      <c r="C60" s="16" t="n"/>
+      <c r="E60" s="17" t="n"/>
+      <c r="F60" s="18" t="n"/>
+      <c r="G60" s="19" t="n"/>
+      <c r="H60" s="20" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="n"/>
+      <c r="B61" s="15" t="n"/>
+      <c r="C61" s="16" t="n"/>
+      <c r="E61" s="17" t="n"/>
+      <c r="F61" s="18" t="n"/>
+      <c r="G61" s="19" t="n"/>
+      <c r="H61" s="20" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="n"/>
+      <c r="B62" s="15" t="n"/>
+      <c r="C62" s="16" t="n"/>
+      <c r="E62" s="17" t="n"/>
+      <c r="F62" s="18" t="n"/>
+      <c r="G62" s="19" t="n"/>
+      <c r="H62" s="20" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="n"/>
+      <c r="B63" s="15" t="n"/>
+      <c r="C63" s="16" t="n"/>
+      <c r="E63" s="17" t="n"/>
+      <c r="F63" s="18" t="n"/>
+      <c r="G63" s="19" t="n"/>
+      <c r="H63" s="20" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="n"/>
+      <c r="B64" s="15" t="n"/>
+      <c r="C64" s="16" t="n"/>
+      <c r="E64" s="17" t="n"/>
+      <c r="F64" s="18" t="n"/>
+      <c r="G64" s="19" t="n"/>
+      <c r="H64" s="20" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="n"/>
+      <c r="B65" s="15" t="n"/>
+      <c r="C65" s="16" t="n"/>
+      <c r="E65" s="17" t="n"/>
+      <c r="F65" s="18" t="n"/>
+      <c r="G65" s="19" t="n"/>
+      <c r="H65" s="20" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="n"/>
+      <c r="B66" s="15" t="n"/>
+      <c r="C66" s="16" t="n"/>
+      <c r="E66" s="17" t="n"/>
+      <c r="F66" s="18" t="n"/>
+      <c r="G66" s="19" t="n"/>
+      <c r="H66" s="20" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="n"/>
+      <c r="B67" s="15" t="n"/>
+      <c r="C67" s="16" t="n"/>
+      <c r="E67" s="17" t="n"/>
+      <c r="F67" s="18" t="n"/>
+      <c r="G67" s="19" t="n"/>
+      <c r="H67" s="20" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="21" t="inlineStr">
+        <is>
+          <t>RIEPILOGO MENSILE (calcolato in automatico dalla colonna Data)</t>
+        </is>
+      </c>
+      <c r="E70" s="22" t="inlineStr">
+        <is>
+          <t>Nota: le righe senza data entrano nei totali generali ma non nel mese.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="23" t="inlineStr">
+        <is>
+          <t>Mese</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>Costi (netto IVA)</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>Ricavi (netto IVA)</t>
+        </is>
+      </c>
+      <c r="E71" s="23" t="inlineStr">
+        <is>
+          <t>Utile / Perdita</t>
+        </is>
+      </c>
+      <c r="F71" s="23" t="inlineStr">
+        <is>
+          <t>Corsi venduti</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="24">
+        <f>DATE(2026,10,1)</f>
+        <v/>
+      </c>
+      <c r="B72" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A72,$A$8:$A$67,"&lt;"&amp;EDATE(A72,1))</f>
+        <v/>
+      </c>
+      <c r="C72" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A72,$E$8:$E$67,"&lt;"&amp;EDATE(A72,1))</f>
+        <v/>
+      </c>
+      <c r="E72" s="27">
+        <f>C72-B72</f>
+        <v/>
+      </c>
+      <c r="F72" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A72,$E$8:$E$67,"&lt;"&amp;EDATE(A72,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="24">
+        <f>EDATE(A72,1)</f>
+        <v/>
+      </c>
+      <c r="B73" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A73,$A$8:$A$67,"&lt;"&amp;EDATE(A73,1))</f>
+        <v/>
+      </c>
+      <c r="C73" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A73,$E$8:$E$67,"&lt;"&amp;EDATE(A73,1))</f>
+        <v/>
+      </c>
+      <c r="E73" s="27">
+        <f>C73-B73</f>
+        <v/>
+      </c>
+      <c r="F73" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A73,$E$8:$E$67,"&lt;"&amp;EDATE(A73,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="24">
+        <f>EDATE(A73,1)</f>
+        <v/>
+      </c>
+      <c r="B74" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A74,$A$8:$A$67,"&lt;"&amp;EDATE(A74,1))</f>
+        <v/>
+      </c>
+      <c r="C74" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A74,$E$8:$E$67,"&lt;"&amp;EDATE(A74,1))</f>
+        <v/>
+      </c>
+      <c r="E74" s="27">
+        <f>C74-B74</f>
+        <v/>
+      </c>
+      <c r="F74" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A74,$E$8:$E$67,"&lt;"&amp;EDATE(A74,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="24">
+        <f>EDATE(A74,1)</f>
+        <v/>
+      </c>
+      <c r="B75" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A75,$A$8:$A$67,"&lt;"&amp;EDATE(A75,1))</f>
+        <v/>
+      </c>
+      <c r="C75" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A75,$E$8:$E$67,"&lt;"&amp;EDATE(A75,1))</f>
+        <v/>
+      </c>
+      <c r="E75" s="27">
+        <f>C75-B75</f>
+        <v/>
+      </c>
+      <c r="F75" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A75,$E$8:$E$67,"&lt;"&amp;EDATE(A75,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="24">
+        <f>EDATE(A75,1)</f>
+        <v/>
+      </c>
+      <c r="B76" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A76,$A$8:$A$67,"&lt;"&amp;EDATE(A76,1))</f>
+        <v/>
+      </c>
+      <c r="C76" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A76,$E$8:$E$67,"&lt;"&amp;EDATE(A76,1))</f>
+        <v/>
+      </c>
+      <c r="E76" s="27">
+        <f>C76-B76</f>
+        <v/>
+      </c>
+      <c r="F76" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A76,$E$8:$E$67,"&lt;"&amp;EDATE(A76,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="24">
+        <f>EDATE(A76,1)</f>
+        <v/>
+      </c>
+      <c r="B77" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A77,$A$8:$A$67,"&lt;"&amp;EDATE(A77,1))</f>
+        <v/>
+      </c>
+      <c r="C77" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A77,$E$8:$E$67,"&lt;"&amp;EDATE(A77,1))</f>
+        <v/>
+      </c>
+      <c r="E77" s="27">
+        <f>C77-B77</f>
+        <v/>
+      </c>
+      <c r="F77" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A77,$E$8:$E$67,"&lt;"&amp;EDATE(A77,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="24">
+        <f>EDATE(A77,1)</f>
+        <v/>
+      </c>
+      <c r="B78" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A78,$A$8:$A$67,"&lt;"&amp;EDATE(A78,1))</f>
+        <v/>
+      </c>
+      <c r="C78" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A78,$E$8:$E$67,"&lt;"&amp;EDATE(A78,1))</f>
+        <v/>
+      </c>
+      <c r="E78" s="27">
+        <f>C78-B78</f>
+        <v/>
+      </c>
+      <c r="F78" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A78,$E$8:$E$67,"&lt;"&amp;EDATE(A78,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="24">
+        <f>EDATE(A78,1)</f>
+        <v/>
+      </c>
+      <c r="B79" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A79,$A$8:$A$67,"&lt;"&amp;EDATE(A79,1))</f>
+        <v/>
+      </c>
+      <c r="C79" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A79,$E$8:$E$67,"&lt;"&amp;EDATE(A79,1))</f>
+        <v/>
+      </c>
+      <c r="E79" s="27">
+        <f>C79-B79</f>
+        <v/>
+      </c>
+      <c r="F79" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A79,$E$8:$E$67,"&lt;"&amp;EDATE(A79,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="24">
+        <f>EDATE(A79,1)</f>
+        <v/>
+      </c>
+      <c r="B80" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A80,$A$8:$A$67,"&lt;"&amp;EDATE(A80,1))</f>
+        <v/>
+      </c>
+      <c r="C80" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A80,$E$8:$E$67,"&lt;"&amp;EDATE(A80,1))</f>
+        <v/>
+      </c>
+      <c r="E80" s="27">
+        <f>C80-B80</f>
+        <v/>
+      </c>
+      <c r="F80" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A80,$E$8:$E$67,"&lt;"&amp;EDATE(A80,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="24">
+        <f>EDATE(A80,1)</f>
+        <v/>
+      </c>
+      <c r="B81" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A81,$A$8:$A$67,"&lt;"&amp;EDATE(A81,1))</f>
+        <v/>
+      </c>
+      <c r="C81" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A81,$E$8:$E$67,"&lt;"&amp;EDATE(A81,1))</f>
+        <v/>
+      </c>
+      <c r="E81" s="27">
+        <f>C81-B81</f>
+        <v/>
+      </c>
+      <c r="F81" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A81,$E$8:$E$67,"&lt;"&amp;EDATE(A81,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="24">
+        <f>EDATE(A81,1)</f>
+        <v/>
+      </c>
+      <c r="B82" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A82,$A$8:$A$67,"&lt;"&amp;EDATE(A82,1))</f>
+        <v/>
+      </c>
+      <c r="C82" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A82,$E$8:$E$67,"&lt;"&amp;EDATE(A82,1))</f>
+        <v/>
+      </c>
+      <c r="E82" s="27">
+        <f>C82-B82</f>
+        <v/>
+      </c>
+      <c r="F82" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A82,$E$8:$E$67,"&lt;"&amp;EDATE(A82,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="24">
+        <f>EDATE(A82,1)</f>
+        <v/>
+      </c>
+      <c r="B83" s="25">
+        <f>SUMIFS($C$8:$C$67,$A$8:$A$67,"&gt;="&amp;A83,$A$8:$A$67,"&lt;"&amp;EDATE(A83,1))</f>
+        <v/>
+      </c>
+      <c r="C83" s="26">
+        <f>SUMIFS($H$8:$H$67,$E$8:$E$67,"&gt;="&amp;A83,$E$8:$E$67,"&lt;"&amp;EDATE(A83,1))</f>
+        <v/>
+      </c>
+      <c r="E83" s="27">
+        <f>C83-B83</f>
+        <v/>
+      </c>
+      <c r="F83" s="28">
+        <f>SUMIFS($G$8:$G$67,$E$8:$E$67,"&gt;="&amp;A83,$E$8:$E$67,"&lt;"&amp;EDATE(A83,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>TOTALE</t>
+        </is>
+      </c>
+      <c r="B84" s="30">
+        <f>SUM(B72:B83)</f>
+        <v/>
+      </c>
+      <c r="C84" s="30">
+        <f>SUM(C72:C83)</f>
+        <v/>
+      </c>
+      <c r="E84" s="31">
+        <f>C84-B84</f>
+        <v/>
+      </c>
+      <c r="F84" s="32">
+        <f>SUM(F72:F83)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A70:D70"/>
+    <mergeCell ref="E70:H70"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A6:B6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C8:C37 H8:H37" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Importo non valido" error="Inserire un importo positivo, AL NETTO DI IVA." promptTitle="Al netto di IVA" prompt="Inserire l'importo SENZA IVA." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="C8:C67 H8:H67" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Importo non valido" error="Inserire un importo positivo, AL NETTO DI IVA." promptTitle="Al netto di IVA" prompt="Inserire l'importo SENZA IVA." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Excel corso invalidità civile: aggiungi ricavi da downselling (registrazione del corso)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UJqD5pkzvn9qNWWBae35Bo
</commit_message>
<xml_diff>
--- a/Corso_Invalidita_Civile_Ottobre_2026.xlsx
+++ b/Corso_Invalidita_Civile_Ottobre_2026.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costi e Ricavi" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Costi e Ricavi'!$A$1:$F$74</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Costi e Ricavi'!$A$1:$F$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,14 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00 &quot;€&quot;;-#,##0.00 &quot;€&quot;"/>
-    <numFmt numFmtId="167" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="168" formatCode="MMMM YYYY"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="167" formatCode="MMMM YYYY"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +60,24 @@
       <sz val="12"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="002E7D32"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00558B2F"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00558B2F"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00000000"/>
     </font>
@@ -75,13 +92,13 @@
       <sz val="16"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
       <i val="1"/>
       <color rgb="007F7F7F"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
@@ -170,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -193,51 +210,66 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="19" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <b val="1"/>
@@ -269,6 +301,17 @@
         <patternFill patternType="solid">
           <fgColor rgb="00E3F4E4"/>
           <bgColor rgb="00E3F4E4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00558B2F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F3F9E8"/>
+          <bgColor rgb="00F3F9E8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -634,12 +677,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -666,7 +709,7 @@
         </is>
       </c>
       <c r="E4" s="4">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo")</f>
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo")</f>
         <v/>
       </c>
     </row>
@@ -677,825 +720,871 @@
         </is>
       </c>
       <c r="E5" s="6">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo")</f>
+        <f>E6+E7</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>di cui corso (online e dal vivo)</t>
+        </is>
+      </c>
+      <c r="E6" s="8">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>di cui downselling (registrazione)</t>
+        </is>
+      </c>
+      <c r="E7" s="10">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>UTILE (se ricavi &gt; costi)</t>
         </is>
       </c>
-      <c r="E6" s="6">
+      <c r="E8" s="6">
         <f>MAX(E5-E4,0)</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>PERDITA (se costi &gt; ricavi)</t>
         </is>
       </c>
-      <c r="E7" s="4">
+      <c r="E9" s="4">
         <f>MAX(E4-E5,0)</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>ROI</t>
         </is>
       </c>
-      <c r="E8" s="8">
+      <c r="E10" s="12">
         <f>IF(E4=0,"",(E5-E4)/E4)</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>CORSI VENDUTI</t>
-        </is>
-      </c>
-      <c r="E9" s="9">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="10">
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>CORSI VENDUTI (online e dal vivo)</t>
+        </is>
+      </c>
+      <c r="E11" s="13">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>REGISTRAZIONI VENDUTE (downselling)</t>
+        </is>
+      </c>
+      <c r="E12" s="13">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="14">
         <f>IF(E5&gt;=E4,"RISULTATO FINALE:  UTILE","RISULTATO FINALE:  PERDITA")</f>
         <v/>
       </c>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="12">
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="16">
         <f>ABS(E5-E4)</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="13" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Inserire un movimento per riga: scegliere Costo (sponsorizzate Facebook) o Ricavo (vendita corsi online). La riga si colora da sola.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="17" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="18" t="n"/>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Un movimento per riga. Tipo: Costo (sponsorizzate Facebook), Ricavo corso (online e dal vivo) o Ricavo downselling (registrazione a prezzo ridotto). La riga si colora da sola.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>Tipo
-(Costo / Ricavo)</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>Descrizione</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>N. corsi venduti</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>N. vendite</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
         <is>
           <t>Importo €
 (netto IVA)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="17" t="n"/>
-      <c r="B17" s="18" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="21" t="n"/>
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>Costo</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>Sponsorizzata Facebook</t>
         </is>
       </c>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="20" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="n"/>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Ricavo</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>Vendita corso online</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="20" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="n"/>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="20" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="18" t="n"/>
-      <c r="E20" s="20" t="n"/>
+      <c r="D20" s="22" t="n"/>
+      <c r="E20" s="24" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="n"/>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="20" t="n"/>
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>Ricavo corso</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Vendita corso online / dal vivo</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="24" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="n"/>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="20" t="n"/>
+      <c r="A22" s="21" t="n"/>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Ricavo downselling</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Vendita registrazione del corso</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="24" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="n"/>
-      <c r="B23" s="18" t="n"/>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="20" t="n"/>
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="24" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n"/>
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="20" t="n"/>
+      <c r="A24" s="21" t="n"/>
+      <c r="B24" s="22" t="n"/>
+      <c r="C24" s="23" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="24" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n"/>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="20" t="n"/>
+      <c r="A25" s="21" t="n"/>
+      <c r="B25" s="22" t="n"/>
+      <c r="C25" s="23" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="24" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="n"/>
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="20" t="n"/>
+      <c r="A26" s="21" t="n"/>
+      <c r="B26" s="22" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="24" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="n"/>
-      <c r="B27" s="18" t="n"/>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="20" t="n"/>
+      <c r="A27" s="21" t="n"/>
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="24" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="n"/>
-      <c r="B28" s="18" t="n"/>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="20" t="n"/>
+      <c r="A28" s="21" t="n"/>
+      <c r="B28" s="22" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="24" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="n"/>
-      <c r="B29" s="18" t="n"/>
-      <c r="C29" s="19" t="n"/>
-      <c r="D29" s="18" t="n"/>
-      <c r="E29" s="20" t="n"/>
+      <c r="A29" s="21" t="n"/>
+      <c r="B29" s="22" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="D29" s="22" t="n"/>
+      <c r="E29" s="24" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="n"/>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="20" t="n"/>
+      <c r="A30" s="21" t="n"/>
+      <c r="B30" s="22" t="n"/>
+      <c r="C30" s="23" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="24" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="n"/>
-      <c r="B31" s="18" t="n"/>
-      <c r="C31" s="19" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="20" t="n"/>
+      <c r="A31" s="21" t="n"/>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="23" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="24" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="n"/>
-      <c r="B32" s="18" t="n"/>
-      <c r="C32" s="19" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="20" t="n"/>
+      <c r="A32" s="21" t="n"/>
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="23" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="24" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="n"/>
-      <c r="B33" s="18" t="n"/>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="20" t="n"/>
+      <c r="A33" s="21" t="n"/>
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="23" t="n"/>
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="24" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="n"/>
-      <c r="B34" s="18" t="n"/>
-      <c r="C34" s="19" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="20" t="n"/>
+      <c r="A34" s="21" t="n"/>
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="23" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="24" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="n"/>
-      <c r="B35" s="18" t="n"/>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="18" t="n"/>
-      <c r="E35" s="20" t="n"/>
+      <c r="A35" s="21" t="n"/>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="23" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="24" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="n"/>
-      <c r="B36" s="18" t="n"/>
-      <c r="C36" s="19" t="n"/>
-      <c r="D36" s="18" t="n"/>
-      <c r="E36" s="20" t="n"/>
+      <c r="A36" s="21" t="n"/>
+      <c r="B36" s="22" t="n"/>
+      <c r="C36" s="23" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="24" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="n"/>
-      <c r="B37" s="18" t="n"/>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="20" t="n"/>
+      <c r="A37" s="21" t="n"/>
+      <c r="B37" s="22" t="n"/>
+      <c r="C37" s="23" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="24" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="n"/>
-      <c r="B38" s="18" t="n"/>
-      <c r="C38" s="19" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="20" t="n"/>
+      <c r="A38" s="21" t="n"/>
+      <c r="B38" s="22" t="n"/>
+      <c r="C38" s="23" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="24" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="n"/>
-      <c r="B39" s="18" t="n"/>
-      <c r="C39" s="19" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="20" t="n"/>
+      <c r="A39" s="21" t="n"/>
+      <c r="B39" s="22" t="n"/>
+      <c r="C39" s="23" t="n"/>
+      <c r="D39" s="22" t="n"/>
+      <c r="E39" s="24" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="n"/>
-      <c r="B40" s="18" t="n"/>
-      <c r="C40" s="19" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="20" t="n"/>
+      <c r="A40" s="21" t="n"/>
+      <c r="B40" s="22" t="n"/>
+      <c r="C40" s="23" t="n"/>
+      <c r="D40" s="22" t="n"/>
+      <c r="E40" s="24" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="n"/>
-      <c r="B41" s="18" t="n"/>
-      <c r="C41" s="19" t="n"/>
-      <c r="D41" s="18" t="n"/>
-      <c r="E41" s="20" t="n"/>
+      <c r="A41" s="21" t="n"/>
+      <c r="B41" s="22" t="n"/>
+      <c r="C41" s="23" t="n"/>
+      <c r="D41" s="22" t="n"/>
+      <c r="E41" s="24" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="n"/>
-      <c r="B42" s="18" t="n"/>
-      <c r="C42" s="19" t="n"/>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="20" t="n"/>
+      <c r="A42" s="21" t="n"/>
+      <c r="B42" s="22" t="n"/>
+      <c r="C42" s="23" t="n"/>
+      <c r="D42" s="22" t="n"/>
+      <c r="E42" s="24" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="n"/>
-      <c r="B43" s="18" t="n"/>
-      <c r="C43" s="19" t="n"/>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="20" t="n"/>
+      <c r="A43" s="21" t="n"/>
+      <c r="B43" s="22" t="n"/>
+      <c r="C43" s="23" t="n"/>
+      <c r="D43" s="22" t="n"/>
+      <c r="E43" s="24" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="n"/>
-      <c r="B44" s="18" t="n"/>
-      <c r="C44" s="19" t="n"/>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="20" t="n"/>
+      <c r="A44" s="21" t="n"/>
+      <c r="B44" s="22" t="n"/>
+      <c r="C44" s="23" t="n"/>
+      <c r="D44" s="22" t="n"/>
+      <c r="E44" s="24" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="n"/>
-      <c r="B45" s="18" t="n"/>
-      <c r="C45" s="19" t="n"/>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="20" t="n"/>
+      <c r="A45" s="21" t="n"/>
+      <c r="B45" s="22" t="n"/>
+      <c r="C45" s="23" t="n"/>
+      <c r="D45" s="22" t="n"/>
+      <c r="E45" s="24" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="n"/>
-      <c r="B46" s="18" t="n"/>
-      <c r="C46" s="19" t="n"/>
-      <c r="D46" s="18" t="n"/>
-      <c r="E46" s="20" t="n"/>
+      <c r="A46" s="21" t="n"/>
+      <c r="B46" s="22" t="n"/>
+      <c r="C46" s="23" t="n"/>
+      <c r="D46" s="22" t="n"/>
+      <c r="E46" s="24" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="n"/>
-      <c r="B47" s="18" t="n"/>
-      <c r="C47" s="19" t="n"/>
-      <c r="D47" s="18" t="n"/>
-      <c r="E47" s="20" t="n"/>
+      <c r="A47" s="21" t="n"/>
+      <c r="B47" s="22" t="n"/>
+      <c r="C47" s="23" t="n"/>
+      <c r="D47" s="22" t="n"/>
+      <c r="E47" s="24" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="n"/>
-      <c r="B48" s="18" t="n"/>
-      <c r="C48" s="19" t="n"/>
-      <c r="D48" s="18" t="n"/>
-      <c r="E48" s="20" t="n"/>
+      <c r="A48" s="21" t="n"/>
+      <c r="B48" s="22" t="n"/>
+      <c r="C48" s="23" t="n"/>
+      <c r="D48" s="22" t="n"/>
+      <c r="E48" s="24" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="n"/>
-      <c r="B49" s="18" t="n"/>
-      <c r="C49" s="19" t="n"/>
-      <c r="D49" s="18" t="n"/>
-      <c r="E49" s="20" t="n"/>
+      <c r="A49" s="21" t="n"/>
+      <c r="B49" s="22" t="n"/>
+      <c r="C49" s="23" t="n"/>
+      <c r="D49" s="22" t="n"/>
+      <c r="E49" s="24" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="17" t="n"/>
-      <c r="B50" s="18" t="n"/>
-      <c r="C50" s="19" t="n"/>
-      <c r="D50" s="18" t="n"/>
-      <c r="E50" s="20" t="n"/>
+      <c r="A50" s="21" t="n"/>
+      <c r="B50" s="22" t="n"/>
+      <c r="C50" s="23" t="n"/>
+      <c r="D50" s="22" t="n"/>
+      <c r="E50" s="24" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="n"/>
-      <c r="B51" s="18" t="n"/>
-      <c r="C51" s="19" t="n"/>
-      <c r="D51" s="18" t="n"/>
-      <c r="E51" s="20" t="n"/>
+      <c r="A51" s="21" t="n"/>
+      <c r="B51" s="22" t="n"/>
+      <c r="C51" s="23" t="n"/>
+      <c r="D51" s="22" t="n"/>
+      <c r="E51" s="24" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="n"/>
-      <c r="B52" s="18" t="n"/>
-      <c r="C52" s="19" t="n"/>
-      <c r="D52" s="18" t="n"/>
-      <c r="E52" s="20" t="n"/>
+      <c r="A52" s="21" t="n"/>
+      <c r="B52" s="22" t="n"/>
+      <c r="C52" s="23" t="n"/>
+      <c r="D52" s="22" t="n"/>
+      <c r="E52" s="24" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="17" t="n"/>
-      <c r="B53" s="18" t="n"/>
-      <c r="C53" s="19" t="n"/>
-      <c r="D53" s="18" t="n"/>
-      <c r="E53" s="20" t="n"/>
+      <c r="A53" s="21" t="n"/>
+      <c r="B53" s="22" t="n"/>
+      <c r="C53" s="23" t="n"/>
+      <c r="D53" s="22" t="n"/>
+      <c r="E53" s="24" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="17" t="n"/>
-      <c r="B54" s="18" t="n"/>
-      <c r="C54" s="19" t="n"/>
-      <c r="D54" s="18" t="n"/>
-      <c r="E54" s="20" t="n"/>
+      <c r="A54" s="21" t="n"/>
+      <c r="B54" s="22" t="n"/>
+      <c r="C54" s="23" t="n"/>
+      <c r="D54" s="22" t="n"/>
+      <c r="E54" s="24" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="n"/>
-      <c r="B55" s="18" t="n"/>
-      <c r="C55" s="19" t="n"/>
-      <c r="D55" s="18" t="n"/>
-      <c r="E55" s="20" t="n"/>
+      <c r="A55" s="21" t="n"/>
+      <c r="B55" s="22" t="n"/>
+      <c r="C55" s="23" t="n"/>
+      <c r="D55" s="22" t="n"/>
+      <c r="E55" s="24" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="17" t="n"/>
-      <c r="B56" s="18" t="n"/>
-      <c r="C56" s="19" t="n"/>
-      <c r="D56" s="18" t="n"/>
-      <c r="E56" s="20" t="n"/>
+      <c r="A56" s="21" t="n"/>
+      <c r="B56" s="22" t="n"/>
+      <c r="C56" s="23" t="n"/>
+      <c r="D56" s="22" t="n"/>
+      <c r="E56" s="24" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="21" t="n"/>
+      <c r="B57" s="22" t="n"/>
+      <c r="C57" s="23" t="n"/>
+      <c r="D57" s="22" t="n"/>
+      <c r="E57" s="24" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="21" t="n"/>
+      <c r="B58" s="22" t="n"/>
+      <c r="C58" s="23" t="n"/>
+      <c r="D58" s="22" t="n"/>
+      <c r="E58" s="24" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="21" t="inlineStr">
+      <c r="A59" s="21" t="n"/>
+      <c r="B59" s="22" t="n"/>
+      <c r="C59" s="23" t="n"/>
+      <c r="D59" s="22" t="n"/>
+      <c r="E59" s="24" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
         <is>
           <t>RIEPILOGO MENSILE (calcolato in automatico dalla colonna Data)</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="15" t="inlineStr">
-        <is>
-          <t>Nota: le righe senza data entrano nei totali generali ma non nel mese.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="16" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>Nota: le righe senza data entrano nei totali generali ma non nel mese. Ricavi = corso + downselling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="20" t="inlineStr">
         <is>
           <t>Mese</t>
         </is>
       </c>
-      <c r="B61" s="22" t="inlineStr">
+      <c r="B64" s="27" t="inlineStr">
         <is>
           <t>Costi (netto IVA)</t>
         </is>
       </c>
-      <c r="C61" s="23" t="inlineStr">
+      <c r="C64" s="28" t="inlineStr">
         <is>
           <t>Ricavi (netto IVA)</t>
         </is>
       </c>
-      <c r="D61" s="23" t="inlineStr">
+      <c r="D64" s="28" t="inlineStr">
         <is>
           <t>Utile</t>
         </is>
       </c>
-      <c r="E61" s="22" t="inlineStr">
+      <c r="E64" s="27" t="inlineStr">
         <is>
           <t>Perdita</t>
         </is>
       </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>Corsi venduti</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="24">
+      <c r="F64" s="20" t="inlineStr">
+        <is>
+          <t>N. vendite</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="29">
         <f>DATE(2026,10,1)</f>
         <v/>
       </c>
-      <c r="B62" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A62,$A$17:$A$56,"&lt;"&amp;EDATE(A62,1))</f>
-        <v/>
-      </c>
-      <c r="C62" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A62,$A$17:$A$56,"&lt;"&amp;EDATE(A62,1))</f>
-        <v/>
-      </c>
-      <c r="D62" s="26">
-        <f>MAX(C62-B62,0)</f>
-        <v/>
-      </c>
-      <c r="E62" s="25">
-        <f>MAX(B62-C62,0)</f>
-        <v/>
-      </c>
-      <c r="F62" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A62,$A$17:$A$56,"&lt;"&amp;EDATE(A62,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="24">
-        <f>EDATE(A62,1)</f>
-        <v/>
-      </c>
-      <c r="B63" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A63,$A$17:$A$56,"&lt;"&amp;EDATE(A63,1))</f>
-        <v/>
-      </c>
-      <c r="C63" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A63,$A$17:$A$56,"&lt;"&amp;EDATE(A63,1))</f>
-        <v/>
-      </c>
-      <c r="D63" s="26">
-        <f>MAX(C63-B63,0)</f>
-        <v/>
-      </c>
-      <c r="E63" s="25">
-        <f>MAX(B63-C63,0)</f>
-        <v/>
-      </c>
-      <c r="F63" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A63,$A$17:$A$56,"&lt;"&amp;EDATE(A63,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="24">
-        <f>EDATE(A63,1)</f>
-        <v/>
-      </c>
-      <c r="B64" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A64,$A$17:$A$56,"&lt;"&amp;EDATE(A64,1))</f>
-        <v/>
-      </c>
-      <c r="C64" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A64,$A$17:$A$56,"&lt;"&amp;EDATE(A64,1))</f>
-        <v/>
-      </c>
-      <c r="D64" s="26">
-        <f>MAX(C64-B64,0)</f>
-        <v/>
-      </c>
-      <c r="E64" s="25">
-        <f>MAX(B64-C64,0)</f>
-        <v/>
-      </c>
-      <c r="F64" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A64,$A$17:$A$56,"&lt;"&amp;EDATE(A64,1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="24">
-        <f>EDATE(A64,1)</f>
-        <v/>
-      </c>
-      <c r="B65" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A65,$A$17:$A$56,"&lt;"&amp;EDATE(A65,1))</f>
-        <v/>
-      </c>
-      <c r="C65" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A65,$A$17:$A$56,"&lt;"&amp;EDATE(A65,1))</f>
-        <v/>
-      </c>
-      <c r="D65" s="26">
+      <c r="B65" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A65,$A$20:$A$59,"&lt;"&amp;EDATE(A65,1))</f>
+        <v/>
+      </c>
+      <c r="C65" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A65,$A$20:$A$59,"&lt;"&amp;EDATE(A65,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A65,$A$20:$A$59,"&lt;"&amp;EDATE(A65,1))</f>
+        <v/>
+      </c>
+      <c r="D65" s="31">
         <f>MAX(C65-B65,0)</f>
         <v/>
       </c>
-      <c r="E65" s="25">
+      <c r="E65" s="30">
         <f>MAX(B65-C65,0)</f>
         <v/>
       </c>
-      <c r="F65" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A65,$A$17:$A$56,"&lt;"&amp;EDATE(A65,1))</f>
+      <c r="F65" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A65,$A$20:$A$59,"&lt;"&amp;EDATE(A65,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A65,$A$20:$A$59,"&lt;"&amp;EDATE(A65,1))</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="24">
+      <c r="A66" s="29">
         <f>EDATE(A65,1)</f>
         <v/>
       </c>
-      <c r="B66" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A66,$A$17:$A$56,"&lt;"&amp;EDATE(A66,1))</f>
-        <v/>
-      </c>
-      <c r="C66" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A66,$A$17:$A$56,"&lt;"&amp;EDATE(A66,1))</f>
-        <v/>
-      </c>
-      <c r="D66" s="26">
+      <c r="B66" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A66,$A$20:$A$59,"&lt;"&amp;EDATE(A66,1))</f>
+        <v/>
+      </c>
+      <c r="C66" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A66,$A$20:$A$59,"&lt;"&amp;EDATE(A66,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A66,$A$20:$A$59,"&lt;"&amp;EDATE(A66,1))</f>
+        <v/>
+      </c>
+      <c r="D66" s="31">
         <f>MAX(C66-B66,0)</f>
         <v/>
       </c>
-      <c r="E66" s="25">
+      <c r="E66" s="30">
         <f>MAX(B66-C66,0)</f>
         <v/>
       </c>
-      <c r="F66" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A66,$A$17:$A$56,"&lt;"&amp;EDATE(A66,1))</f>
+      <c r="F66" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A66,$A$20:$A$59,"&lt;"&amp;EDATE(A66,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A66,$A$20:$A$59,"&lt;"&amp;EDATE(A66,1))</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="24">
+      <c r="A67" s="29">
         <f>EDATE(A66,1)</f>
         <v/>
       </c>
-      <c r="B67" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A67,$A$17:$A$56,"&lt;"&amp;EDATE(A67,1))</f>
-        <v/>
-      </c>
-      <c r="C67" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A67,$A$17:$A$56,"&lt;"&amp;EDATE(A67,1))</f>
-        <v/>
-      </c>
-      <c r="D67" s="26">
+      <c r="B67" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A67,$A$20:$A$59,"&lt;"&amp;EDATE(A67,1))</f>
+        <v/>
+      </c>
+      <c r="C67" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A67,$A$20:$A$59,"&lt;"&amp;EDATE(A67,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A67,$A$20:$A$59,"&lt;"&amp;EDATE(A67,1))</f>
+        <v/>
+      </c>
+      <c r="D67" s="31">
         <f>MAX(C67-B67,0)</f>
         <v/>
       </c>
-      <c r="E67" s="25">
+      <c r="E67" s="30">
         <f>MAX(B67-C67,0)</f>
         <v/>
       </c>
-      <c r="F67" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A67,$A$17:$A$56,"&lt;"&amp;EDATE(A67,1))</f>
+      <c r="F67" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A67,$A$20:$A$59,"&lt;"&amp;EDATE(A67,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A67,$A$20:$A$59,"&lt;"&amp;EDATE(A67,1))</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="24">
+      <c r="A68" s="29">
         <f>EDATE(A67,1)</f>
         <v/>
       </c>
-      <c r="B68" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A68,$A$17:$A$56,"&lt;"&amp;EDATE(A68,1))</f>
-        <v/>
-      </c>
-      <c r="C68" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A68,$A$17:$A$56,"&lt;"&amp;EDATE(A68,1))</f>
-        <v/>
-      </c>
-      <c r="D68" s="26">
+      <c r="B68" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A68,$A$20:$A$59,"&lt;"&amp;EDATE(A68,1))</f>
+        <v/>
+      </c>
+      <c r="C68" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A68,$A$20:$A$59,"&lt;"&amp;EDATE(A68,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A68,$A$20:$A$59,"&lt;"&amp;EDATE(A68,1))</f>
+        <v/>
+      </c>
+      <c r="D68" s="31">
         <f>MAX(C68-B68,0)</f>
         <v/>
       </c>
-      <c r="E68" s="25">
+      <c r="E68" s="30">
         <f>MAX(B68-C68,0)</f>
         <v/>
       </c>
-      <c r="F68" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A68,$A$17:$A$56,"&lt;"&amp;EDATE(A68,1))</f>
+      <c r="F68" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A68,$A$20:$A$59,"&lt;"&amp;EDATE(A68,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A68,$A$20:$A$59,"&lt;"&amp;EDATE(A68,1))</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="24">
+      <c r="A69" s="29">
         <f>EDATE(A68,1)</f>
         <v/>
       </c>
-      <c r="B69" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A69,$A$17:$A$56,"&lt;"&amp;EDATE(A69,1))</f>
-        <v/>
-      </c>
-      <c r="C69" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A69,$A$17:$A$56,"&lt;"&amp;EDATE(A69,1))</f>
-        <v/>
-      </c>
-      <c r="D69" s="26">
+      <c r="B69" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A69,$A$20:$A$59,"&lt;"&amp;EDATE(A69,1))</f>
+        <v/>
+      </c>
+      <c r="C69" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A69,$A$20:$A$59,"&lt;"&amp;EDATE(A69,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A69,$A$20:$A$59,"&lt;"&amp;EDATE(A69,1))</f>
+        <v/>
+      </c>
+      <c r="D69" s="31">
         <f>MAX(C69-B69,0)</f>
         <v/>
       </c>
-      <c r="E69" s="25">
+      <c r="E69" s="30">
         <f>MAX(B69-C69,0)</f>
         <v/>
       </c>
-      <c r="F69" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A69,$A$17:$A$56,"&lt;"&amp;EDATE(A69,1))</f>
+      <c r="F69" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A69,$A$20:$A$59,"&lt;"&amp;EDATE(A69,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A69,$A$20:$A$59,"&lt;"&amp;EDATE(A69,1))</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="24">
+      <c r="A70" s="29">
         <f>EDATE(A69,1)</f>
         <v/>
       </c>
-      <c r="B70" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A70,$A$17:$A$56,"&lt;"&amp;EDATE(A70,1))</f>
-        <v/>
-      </c>
-      <c r="C70" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A70,$A$17:$A$56,"&lt;"&amp;EDATE(A70,1))</f>
-        <v/>
-      </c>
-      <c r="D70" s="26">
+      <c r="B70" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A70,$A$20:$A$59,"&lt;"&amp;EDATE(A70,1))</f>
+        <v/>
+      </c>
+      <c r="C70" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A70,$A$20:$A$59,"&lt;"&amp;EDATE(A70,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A70,$A$20:$A$59,"&lt;"&amp;EDATE(A70,1))</f>
+        <v/>
+      </c>
+      <c r="D70" s="31">
         <f>MAX(C70-B70,0)</f>
         <v/>
       </c>
-      <c r="E70" s="25">
+      <c r="E70" s="30">
         <f>MAX(B70-C70,0)</f>
         <v/>
       </c>
-      <c r="F70" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A70,$A$17:$A$56,"&lt;"&amp;EDATE(A70,1))</f>
+      <c r="F70" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A70,$A$20:$A$59,"&lt;"&amp;EDATE(A70,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A70,$A$20:$A$59,"&lt;"&amp;EDATE(A70,1))</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="24">
+      <c r="A71" s="29">
         <f>EDATE(A70,1)</f>
         <v/>
       </c>
-      <c r="B71" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A71,$A$17:$A$56,"&lt;"&amp;EDATE(A71,1))</f>
-        <v/>
-      </c>
-      <c r="C71" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A71,$A$17:$A$56,"&lt;"&amp;EDATE(A71,1))</f>
-        <v/>
-      </c>
-      <c r="D71" s="26">
+      <c r="B71" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A71,$A$20:$A$59,"&lt;"&amp;EDATE(A71,1))</f>
+        <v/>
+      </c>
+      <c r="C71" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A71,$A$20:$A$59,"&lt;"&amp;EDATE(A71,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A71,$A$20:$A$59,"&lt;"&amp;EDATE(A71,1))</f>
+        <v/>
+      </c>
+      <c r="D71" s="31">
         <f>MAX(C71-B71,0)</f>
         <v/>
       </c>
-      <c r="E71" s="25">
+      <c r="E71" s="30">
         <f>MAX(B71-C71,0)</f>
         <v/>
       </c>
-      <c r="F71" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A71,$A$17:$A$56,"&lt;"&amp;EDATE(A71,1))</f>
+      <c r="F71" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A71,$A$20:$A$59,"&lt;"&amp;EDATE(A71,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A71,$A$20:$A$59,"&lt;"&amp;EDATE(A71,1))</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="24">
+      <c r="A72" s="29">
         <f>EDATE(A71,1)</f>
         <v/>
       </c>
-      <c r="B72" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A72,$A$17:$A$56,"&lt;"&amp;EDATE(A72,1))</f>
-        <v/>
-      </c>
-      <c r="C72" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A72,$A$17:$A$56,"&lt;"&amp;EDATE(A72,1))</f>
-        <v/>
-      </c>
-      <c r="D72" s="26">
+      <c r="B72" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A72,$A$20:$A$59,"&lt;"&amp;EDATE(A72,1))</f>
+        <v/>
+      </c>
+      <c r="C72" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A72,$A$20:$A$59,"&lt;"&amp;EDATE(A72,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A72,$A$20:$A$59,"&lt;"&amp;EDATE(A72,1))</f>
+        <v/>
+      </c>
+      <c r="D72" s="31">
         <f>MAX(C72-B72,0)</f>
         <v/>
       </c>
-      <c r="E72" s="25">
+      <c r="E72" s="30">
         <f>MAX(B72-C72,0)</f>
         <v/>
       </c>
-      <c r="F72" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A72,$A$17:$A$56,"&lt;"&amp;EDATE(A72,1))</f>
+      <c r="F72" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A72,$A$20:$A$59,"&lt;"&amp;EDATE(A72,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A72,$A$20:$A$59,"&lt;"&amp;EDATE(A72,1))</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="24">
+      <c r="A73" s="29">
         <f>EDATE(A72,1)</f>
         <v/>
       </c>
-      <c r="B73" s="25">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Costo",$A$17:$A$56,"&gt;="&amp;A73,$A$17:$A$56,"&lt;"&amp;EDATE(A73,1))</f>
-        <v/>
-      </c>
-      <c r="C73" s="26">
-        <f>SUMIFS($E$17:$E$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A73,$A$17:$A$56,"&lt;"&amp;EDATE(A73,1))</f>
-        <v/>
-      </c>
-      <c r="D73" s="26">
+      <c r="B73" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A73,$A$20:$A$59,"&lt;"&amp;EDATE(A73,1))</f>
+        <v/>
+      </c>
+      <c r="C73" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A73,$A$20:$A$59,"&lt;"&amp;EDATE(A73,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A73,$A$20:$A$59,"&lt;"&amp;EDATE(A73,1))</f>
+        <v/>
+      </c>
+      <c r="D73" s="31">
         <f>MAX(C73-B73,0)</f>
         <v/>
       </c>
-      <c r="E73" s="25">
+      <c r="E73" s="30">
         <f>MAX(B73-C73,0)</f>
         <v/>
       </c>
-      <c r="F73" s="18">
-        <f>SUMIFS($D$17:$D$56,$B$17:$B$56,"Ricavo",$A$17:$A$56,"&gt;="&amp;A73,$A$17:$A$56,"&lt;"&amp;EDATE(A73,1))</f>
+      <c r="F73" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A73,$A$20:$A$59,"&lt;"&amp;EDATE(A73,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A73,$A$20:$A$59,"&lt;"&amp;EDATE(A73,1))</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="27" t="inlineStr">
+      <c r="A74" s="29">
+        <f>EDATE(A73,1)</f>
+        <v/>
+      </c>
+      <c r="B74" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A74,$A$20:$A$59,"&lt;"&amp;EDATE(A74,1))</f>
+        <v/>
+      </c>
+      <c r="C74" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A74,$A$20:$A$59,"&lt;"&amp;EDATE(A74,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A74,$A$20:$A$59,"&lt;"&amp;EDATE(A74,1))</f>
+        <v/>
+      </c>
+      <c r="D74" s="31">
+        <f>MAX(C74-B74,0)</f>
+        <v/>
+      </c>
+      <c r="E74" s="30">
+        <f>MAX(B74-C74,0)</f>
+        <v/>
+      </c>
+      <c r="F74" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A74,$A$20:$A$59,"&lt;"&amp;EDATE(A74,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A74,$A$20:$A$59,"&lt;"&amp;EDATE(A74,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="29">
+        <f>EDATE(A74,1)</f>
+        <v/>
+      </c>
+      <c r="B75" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A75,$A$20:$A$59,"&lt;"&amp;EDATE(A75,1))</f>
+        <v/>
+      </c>
+      <c r="C75" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A75,$A$20:$A$59,"&lt;"&amp;EDATE(A75,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A75,$A$20:$A$59,"&lt;"&amp;EDATE(A75,1))</f>
+        <v/>
+      </c>
+      <c r="D75" s="31">
+        <f>MAX(C75-B75,0)</f>
+        <v/>
+      </c>
+      <c r="E75" s="30">
+        <f>MAX(B75-C75,0)</f>
+        <v/>
+      </c>
+      <c r="F75" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A75,$A$20:$A$59,"&lt;"&amp;EDATE(A75,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A75,$A$20:$A$59,"&lt;"&amp;EDATE(A75,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="29">
+        <f>EDATE(A75,1)</f>
+        <v/>
+      </c>
+      <c r="B76" s="30">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Costo",$A$20:$A$59,"&gt;="&amp;A76,$A$20:$A$59,"&lt;"&amp;EDATE(A76,1))</f>
+        <v/>
+      </c>
+      <c r="C76" s="31">
+        <f>SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A76,$A$20:$A$59,"&lt;"&amp;EDATE(A76,1))+SUMIFS($E$20:$E$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A76,$A$20:$A$59,"&lt;"&amp;EDATE(A76,1))</f>
+        <v/>
+      </c>
+      <c r="D76" s="31">
+        <f>MAX(C76-B76,0)</f>
+        <v/>
+      </c>
+      <c r="E76" s="30">
+        <f>MAX(B76-C76,0)</f>
+        <v/>
+      </c>
+      <c r="F76" s="22">
+        <f>SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo corso",$A$20:$A$59,"&gt;="&amp;A76,$A$20:$A$59,"&lt;"&amp;EDATE(A76,1))+SUMIFS($D$20:$D$59,$B$20:$B$59,"Ricavo downselling",$A$20:$A$59,"&gt;="&amp;A76,$A$20:$A$59,"&lt;"&amp;EDATE(A76,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="32" t="inlineStr">
         <is>
           <t>TOTALE</t>
         </is>
       </c>
-      <c r="B74" s="28">
-        <f>SUM(B62:B73)</f>
-        <v/>
-      </c>
-      <c r="C74" s="28">
-        <f>SUM(C62:C73)</f>
-        <v/>
-      </c>
-      <c r="D74" s="28">
-        <f>MAX(C74-B74,0)</f>
-        <v/>
-      </c>
-      <c r="E74" s="28">
-        <f>MAX(B74-C74,0)</f>
-        <v/>
-      </c>
-      <c r="F74" s="29">
-        <f>SUM(F62:F73)</f>
+      <c r="B77" s="33">
+        <f>SUM(B65:B76)</f>
+        <v/>
+      </c>
+      <c r="C77" s="33">
+        <f>SUM(C65:C76)</f>
+        <v/>
+      </c>
+      <c r="D77" s="33">
+        <f>MAX(C77-B77,0)</f>
+        <v/>
+      </c>
+      <c r="E77" s="33">
+        <f>MAX(B77-C77,0)</f>
+        <v/>
+      </c>
+      <c r="F77" s="34">
+        <f>SUM(F65:F76)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="16">
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A14:D15"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A63:F63"/>
     <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A60:F60"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A11:D12"/>
-    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="E14:E15"/>
   </mergeCells>
-  <conditionalFormatting sqref="A11:E12">
+  <conditionalFormatting sqref="A14:E15">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E$5&lt;$E$4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A17:E56">
+  <conditionalFormatting sqref="A20:E59">
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$B17="Costo"</formula>
+      <formula>$B20="Costo"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>$B17="Ricavo"</formula>
+      <formula>$B20="Ricavo corso"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>$B20="Ricavo downselling"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B17:B56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tipo non valido" error="Scegliere Costo oppure Ricavo dal menu." type="list">
-      <formula1>"Costo,Ricavo"</formula1>
+    <dataValidation sqref="B20:B59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Tipo non valido" error="Scegliere il tipo dal menu." type="list">
+      <formula1>"Costo,Ricavo corso,Ricavo downselling"</formula1>
     </dataValidation>
-    <dataValidation sqref="E17:E56" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Importo non valido" error="Inserire un importo positivo, AL NETTO DI IVA." promptTitle="Al netto di IVA" prompt="Inserire l'importo SENZA IVA." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="E20:E59" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Importo non valido" error="Inserire un importo positivo, AL NETTO DI IVA." promptTitle="Al netto di IVA" prompt="Inserire l'importo SENZA IVA." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>